<commit_message>
docs: log the two-way Mattermost build in the Claude Log sheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AjD4c8Kp1UGQPXfTM8jC9X
</commit_message>
<xml_diff>
--- a/data/Whitewood Family Birthdays.xlsx
+++ b/data/Whitewood Family Birthdays.xlsx
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
   <sheetData>
     <row r="1">
@@ -512,6 +512,34 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>Step 1 live; bot posting confirmed (post 6eyrugxy4byhprobtyo4dc7bpa); awaiting Tyson reply on 10 Sep</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Two-way Mattermost (step 2): bot reads Family Finance, acts on commands/screenshots, answers questions</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Built conversation.py, channel polling, set-up questions, overdue display, direct-debit flag; deployed commits 9438408 and c07ea79. Merged obligations/mattermost/ai keys into the LIVE config file on the server (deploys do not update it). Marked council rates and water as direct debits (Robyn). Fixed the 7am at-job (needed docker exec -i) and posted the September receipts question.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Live test: Tyson asked "what are the last account balances you have on file" at 06:39; bot answered at 09:13 with the six balances. OpenRouter free models: only nvidia/nemotron-3-super-120b-a12b:free answered; free vision models rate-limited, so screenshot reading needs ANTHROPIC_API_KEY in Coolify. Tyson's Mattermost username is tawhai (not dad); allowed_users = tawhai, mum.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Two-way live; awaiting Anthropic key for reliable screenshots; step 3 (phone install) next</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: log the audit and phone-install work in the Claude Log sheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AjD4c8Kp1UGQPXfTM8jC9X
</commit_message>
<xml_diff>
--- a/data/Whitewood Family Birthdays.xlsx
+++ b/data/Whitewood Family Birthdays.xlsx
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
   <sheetData>
     <row r="1">
@@ -540,6 +540,34 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>Two-way live; awaiting Anthropic key for reliable screenshots; step 3 (phone install) next</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Audit the build, add phone install (step 3), confirm two-way Mattermost before bed</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Built the phone install: real PNG icons, service worker with offline page, Obligations as landing page, 180-day login. Independent code review found two real defects, both fixed: a Mattermost failure at 7am used to skip that day for good; an unguarded log write could resend a message or double-count a receipt. Added sqlite WAL and a 30s lock timeout. Deployed commit 7c722dc.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Two-way confirmed live earlier today (bot answered Tyson at 09:13). Reader ran 700+ polls with zero failures. Install: Safari Share &gt; Add to Home Screen; Chrome menu &gt; Install app. Screenshot reading still on free OpenRouter vision models until ANTHROPIC_API_KEY is added.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>All three steps live; 255 tests; next: Anthropic key, then Xero-in-app (step 4) if wanted</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: log the switch to Claude Sonnet 5
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AjD4c8Kp1UGQPXfTM8jC9X
</commit_message>
<xml_diff>
--- a/data/Whitewood Family Birthdays.xlsx
+++ b/data/Whitewood Family Birthdays.xlsx
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
   <sheetData>
     <row r="1">
@@ -568,6 +568,34 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>All three steps live; 255 tests; next: Anthropic key, then Xero-in-app (step 4) if wanted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>46276</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Remove OpenRouter; use Claude Sonnet 5 for all AI</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Deleted every OpenRouter code path (chat, briefing, savings tips, channel answers, screenshot reading). All calls now use the Anthropic SDK with model from config ai.anthropic_model (default claude-sonnet-5). Live config updated. Deployed 9f8cfe1.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Verified on the server: text call answered; a balance image was read correctly (EComm GST $13,129.03). Reader still connected. 256 tests.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Done; screenshots now reliable</t>
         </is>
       </c>
     </row>

</xml_diff>